<commit_message>
Link kritik parça photos to matching sipariş codes in HTML/Excel.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/KRİTİK PARÇA LİSTESİ/Kritik-Parca-Listeleri.xlsx
+++ b/KRİTİK PARÇA LİSTESİ/Kritik-Parca-Listeleri.xlsx
@@ -593,7 +593,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-10-01</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,11 @@
           <t>TERMİK RÖLESİ LR2K0305 0,54-0,8A</t>
         </is>
       </c>
-      <c r="C513" t="inlineStr"/>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>photos/10 00243.jpg</t>
+        </is>
+      </c>
       <c r="D513" t="inlineStr">
         <is>
           <t>Rezistans komple / pano</t>
@@ -3762,7 +3766,11 @@
           <t>TERMİK RÖLESİ LR2K0306 0,80-1,2A</t>
         </is>
       </c>
-      <c r="C514" t="inlineStr"/>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>photos/10 00244.jpg</t>
+        </is>
+      </c>
       <c r="D514" t="inlineStr">
         <is>
           <t>Rezistans komple / pano</t>
@@ -4002,7 +4010,11 @@
           <t>TERMİK RÖLESİ LR2K0314 5,80-8,0A</t>
         </is>
       </c>
-      <c r="C519" t="inlineStr"/>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>photos/10 00249.jpg</t>
+        </is>
+      </c>
       <c r="D519" t="inlineStr">
         <is>
           <t>Rezistans komple / pano</t>
@@ -4098,7 +4110,11 @@
           <t>FAZ KORUMA RÖLESİ MKS-03</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>photos/10 00258.jpg</t>
+        </is>
+      </c>
       <c r="D521" t="inlineStr">
         <is>
           <t>Pano</t>

</xml_diff>

<commit_message>
Add BOM product tree (build_bom, HTML, JSON/CSV) and expand kritik parça data and photos.
Update list HTML, Excel, and build_kritik_sablon pipeline.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/KRİTİK PARÇA LİSTESİ/Kritik-Parca-Listeleri.xlsx
+++ b/KRİTİK PARÇA LİSTESİ/Kritik-Parca-Listeleri.xlsx
@@ -653,7 +653,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -3651,7 +3651,11 @@
           <t>PASLANMAZ SEVİYE BEKÇİSİ</t>
         </is>
       </c>
-      <c r="C509" t="inlineStr"/>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>photos/10 00296.jpg</t>
+        </is>
+      </c>
       <c r="D509" t="inlineStr">
         <is>
           <t>LYM 950–1500</t>
@@ -7998,7 +8002,11 @@
           <t>REZİSTANS 220V 2000W 112CM SERP. DİKİŞSİZ AISI316</t>
         </is>
       </c>
-      <c r="C507" t="inlineStr"/>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>photos/10 07455.jpg</t>
+        </is>
+      </c>
       <c r="D507" t="inlineStr">
         <is>
           <t>VDL 2B 40/50/60/80</t>
@@ -8772,7 +8780,11 @@
           <t>EMİŞ FİLTRESİ KOMPLESİ (PYM2,KBN,VDL,ULT,KNV)</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>photos/07 00670.jpg</t>
+        </is>
+      </c>
       <c r="D521" t="inlineStr">
         <is>
           <t>VDL 1B 40 · VDL 2B 40/50/60/80</t>
@@ -12137,7 +12149,7 @@
       </c>
       <c r="D502" t="inlineStr">
         <is>
-          <t>KBN 1B 1650/1850/2050/2350 · KBN 2B 1650/1850</t>
+          <t>KBN 1B 1650/1850/2050/2350</t>
         </is>
       </c>
       <c r="E502" t="inlineStr">
@@ -12358,10 +12370,14 @@
           <t>REZİSTANS KOMPLESİ 8000W 50CM DÜZ DİKİŞSİZ</t>
         </is>
       </c>
-      <c r="C506" t="inlineStr"/>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>photos/07 15142.jpg</t>
+        </is>
+      </c>
       <c r="D506" t="inlineStr">
         <is>
-          <t>KBN 2B 2050</t>
+          <t>KBN 2B 1650/1850/2050</t>
         </is>
       </c>
       <c r="E506" t="inlineStr">
@@ -13189,7 +13205,11 @@
           <t>POMPA HMSE 40-200/75</t>
         </is>
       </c>
-      <c r="C521" t="inlineStr"/>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>photos/10 17121.jpg</t>
+        </is>
+      </c>
       <c r="D521" t="inlineStr">
         <is>
           <t>KBN 1B 1650/1850</t>
@@ -13560,7 +13580,11 @@
           <t>EMİŞ FİLTRESİ KOMPLESİ (PYM2,KBN,VDL,ULT,KNV)</t>
         </is>
       </c>
-      <c r="C528" t="inlineStr"/>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>photos/07 00670.jpg</t>
+        </is>
+      </c>
       <c r="D528" t="inlineStr">
         <is>
           <t>KBN 1B 1650/1850/2050/2350 · KBN 2B 1650/1850/2050</t>
@@ -14379,7 +14403,11 @@
           <t>PNÖMATİK SİLİNDİR SENSÖRÜ 39CMSE020 CS1E020 CS1-E</t>
         </is>
       </c>
-      <c r="C543" t="inlineStr"/>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>photos/10 05243.jpg</t>
+        </is>
+      </c>
       <c r="D543" t="inlineStr">
         <is>
           <t>KBN 2B 1650/2050</t>
@@ -14432,7 +14460,11 @@
           <t>BASINÇ ŞALTERİ 1-12 BAR 1/4" DS1A3012</t>
         </is>
       </c>
-      <c r="C544" t="inlineStr"/>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>photos/10 16858.jpg</t>
+        </is>
+      </c>
       <c r="D544" t="inlineStr">
         <is>
           <t>KBN 1B 1650 · KBN 2B 1650</t>

</xml_diff>